<commit_message>
scan: seg4 2026-09-29 18:03 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq5_2026-09-29.xlsx
+++ b/output/full_scan/batch_seq5_2026-09-29.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O87"/>
+  <dimension ref="A1:O88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3389,21 +3389,21 @@
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>4441</v>
+        <v>5314</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>振大環球</t>
+          <t>世紀*</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>250.0275992015167</v>
+        <v>258.3112852278673</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>170</v>
+        <v>27.45</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,13 +3414,13 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>37.92821458450216</v>
+        <v>40.33895912445038</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>22.5153089328444</v>
+        <v>16.9305112439531</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>1.163582435675544</v>
+        <v>0.344841567261245</v>
       </c>
       <c r="K56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.2237327614214384</v>
+        <v>-0.4555931304955045</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>4583</v>
+        <v>4441</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>台灣精銳</t>
+          <t>振大環球</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>248.8104155783896</v>
+        <v>250.0275992015167</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>429</v>
+        <v>170</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,13 +3467,13 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>36.63539018502999</v>
+        <v>37.92821458450216</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>27.24875235724973</v>
+        <v>22.5153089328444</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.4894558146914168</v>
+        <v>1.163582435675544</v>
       </c>
       <c r="K57" s="2" t="n">
         <v>0</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>1.994412004920925</v>
+        <v>0.2237327614214384</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3495,21 +3495,21 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>4930</v>
+        <v>4583</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>燦星網</t>
+          <t>台灣精銳</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>248.236997713068</v>
+        <v>248.8104155783896</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>15.85</v>
+        <v>429</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,13 +3520,13 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>42.43203253058726</v>
+        <v>36.63539018502999</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>10.3556392759594</v>
+        <v>27.24875235724973</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.224914502271808</v>
+        <v>0.4894558146914168</v>
       </c>
       <c r="K58" s="2" t="n">
         <v>0</v>
@@ -3538,31 +3538,31 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-0.003768815758597</v>
+        <v>1.994412004920925</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>5871</v>
+        <v>4930</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>中租-KY</t>
+          <t>燦星網</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>241.773435145806</v>
+        <v>248.236997713068</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>107</v>
+        <v>15.85</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,13 +3573,13 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>36.96293586602814</v>
+        <v>42.43203253058726</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>13.38031224713081</v>
+        <v>10.3556392759594</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.6843988788339931</v>
+        <v>0.224914502271808</v>
       </c>
       <c r="K59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.5811092879674181</v>
+        <v>-0.003768815758597</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>5007</v>
+        <v>5871</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>三星</t>
+          <t>中租-KY</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>236.9802237700532</v>
+        <v>241.773435145806</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>55.4</v>
+        <v>107</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,13 +3626,13 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>41.8016438763921</v>
+        <v>36.96293586602814</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>20.20857423028172</v>
+        <v>13.38031224713081</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.9475877364936768</v>
+        <v>0.6843988788339931</v>
       </c>
       <c r="K60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.0376202455204438</v>
+        <v>-0.5811092879674181</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>4766</v>
+        <v>5007</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>南寶</t>
+          <t>三星</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>236.9383567973334</v>
+        <v>236.9802237700532</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>341</v>
+        <v>55.4</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,13 +3679,13 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>50.10510438273813</v>
+        <v>41.8016438763921</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>10.46983093942789</v>
+        <v>20.20857423028172</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.6190949040470715</v>
+        <v>0.9475877364936768</v>
       </c>
       <c r="K61" s="2" t="n">
         <v>0</v>
@@ -3697,31 +3697,31 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-0.0251691969917847</v>
+        <v>-0.0376202455204438</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>5288</v>
+        <v>4766</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>豐祥-KY</t>
+          <t>南寶</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>221.7530792525884</v>
+        <v>236.9383567973334</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>186.5</v>
+        <v>341</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,13 +3732,13 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>48.04860252252803</v>
+        <v>50.10510438273813</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>10.48080451352173</v>
+        <v>10.46983093942789</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.9312042264145488</v>
+        <v>0.6190949040470715</v>
       </c>
       <c r="K62" s="2" t="n">
         <v>0</v>
@@ -3750,31 +3750,31 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.297719828101239</v>
+        <v>-0.0251691969917847</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>6151</v>
+        <v>5288</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>晉倫</t>
+          <t>豐祥-KY</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>219.1720383965921</v>
+        <v>221.7530792525884</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>34.75</v>
+        <v>186.5</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,13 +3785,13 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>44.0732838642881</v>
+        <v>48.04860252252803</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>17.27396938310246</v>
+        <v>10.48080451352173</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.9844075577305456</v>
+        <v>0.9312042264145488</v>
       </c>
       <c r="K63" s="2" t="n">
         <v>0</v>
@@ -3803,31 +3803,31 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.07998107463101781</v>
+        <v>0.297719828101239</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>6146</v>
+        <v>6151</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>耕興</t>
+          <t>晉倫</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>218.6773372799274</v>
+        <v>219.1720383965921</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>180</v>
+        <v>34.75</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,16 +3838,16 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>40.89114082515854</v>
+        <v>44.0732838642881</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>24.96872677764892</v>
+        <v>17.27396938310246</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.5842244339836155</v>
+        <v>0.9844075577305456</v>
       </c>
       <c r="K64" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L64" s="2" t="n">
         <v>0</v>
@@ -3856,31 +3856,31 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.4470953691415502</v>
+        <v>0.07998107463101781</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>4555</v>
+        <v>6146</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>氣立</t>
+          <t>耕興</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>218.3756759246901</v>
+        <v>218.6773372799274</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>41.6</v>
+        <v>180</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,16 +3891,16 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>37.80273892689825</v>
+        <v>40.89114082515854</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>16.32540730130954</v>
+        <v>24.96872677764892</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.5755730232952802</v>
+        <v>0.5842244339836155</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L65" s="2" t="n">
         <v>0</v>
@@ -3909,31 +3909,31 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-0.06958869745328131</v>
+        <v>0.4470953691415502</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>4564</v>
+        <v>4555</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>元翎</t>
+          <t>氣立</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>217.5661937052387</v>
+        <v>218.3756759246901</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>16.2</v>
+        <v>41.6</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,13 +3944,13 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>49.33273210169873</v>
+        <v>37.80273892689825</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>9.849913934296399</v>
+        <v>16.32540730130954</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.7285320044006097</v>
+        <v>0.5755730232952802</v>
       </c>
       <c r="K66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.0756965467895812</v>
+        <v>-0.06958869745328131</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>5519</v>
+        <v>4564</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>隆大</t>
+          <t>元翎</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>216.2273951877729</v>
+        <v>217.5661937052387</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>25</v>
+        <v>16.2</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,13 +3997,13 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>28.69285433830632</v>
+        <v>49.33273210169873</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>36.23236693039034</v>
+        <v>9.849913934296399</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.4616835518987857</v>
+        <v>0.7285320044006097</v>
       </c>
       <c r="K67" s="2" t="n">
         <v>0</v>
@@ -4015,31 +4015,31 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-0.0229854499746738</v>
+        <v>0.0756965467895812</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>4552</v>
+        <v>5519</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>力達-KY</t>
+          <t>隆大</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>213.5729923217325</v>
+        <v>216.2273951877729</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>15.35</v>
+        <v>25</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,13 +4050,13 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>30.1809626714882</v>
+        <v>28.69285433830632</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>41.14055730368716</v>
+        <v>36.23236693039034</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.7021184039246593</v>
+        <v>0.4616835518987857</v>
       </c>
       <c r="K68" s="2" t="n">
         <v>0</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>0.0311982730824437</v>
+        <v>-0.0229854499746738</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4078,21 +4078,21 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>4755</v>
+        <v>4552</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>三福化</t>
+          <t>力達-KY</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>210.2176853678628</v>
+        <v>213.5729923217325</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>118</v>
+        <v>15.35</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,13 +4103,13 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>56.00831438815404</v>
+        <v>30.1809626714882</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>9.207597434980828</v>
+        <v>41.14055730368716</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>1.217377231239728</v>
+        <v>0.7021184039246593</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>0</v>
@@ -4121,31 +4121,31 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.5775206016738379</v>
+        <v>0.0311982730824437</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>4178</v>
+        <v>4755</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>永笙-KY</t>
+          <t>三福化</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>198.2844730846306</v>
+        <v>210.2176853678628</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>16.55</v>
+        <v>118</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,13 +4156,13 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>42.14584275595406</v>
+        <v>56.00831438815404</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>14.32824644836467</v>
+        <v>9.207597434980828</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>1.036365383339548</v>
+        <v>1.217377231239728</v>
       </c>
       <c r="K70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.0240957435038148</v>
+        <v>0.5775206016738379</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>6024</v>
+        <v>4178</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>群益期</t>
+          <t>永笙-KY</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>197.3485839563371</v>
+        <v>198.2844730846306</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>60.2</v>
+        <v>16.55</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,13 +4209,13 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>40.23191530909575</v>
+        <v>42.14584275595406</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>13.07731025224123</v>
+        <v>14.32824644836467</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>1.042909212674573</v>
+        <v>1.036365383339548</v>
       </c>
       <c r="K71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>-0.1005057949140373</v>
+        <v>0.0240957435038148</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>5534</v>
+        <v>6024</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>長虹</t>
+          <t>群益期</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>178.240771971022</v>
+        <v>197.3485839563371</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>73.3</v>
+        <v>60.2</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,13 +4262,13 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>38.58221477615712</v>
+        <v>40.23191530909575</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>16.17922227485474</v>
+        <v>13.07731025224123</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.8600740304657295</v>
+        <v>1.042909212674573</v>
       </c>
       <c r="K72" s="2" t="n">
         <v>0</v>
@@ -4280,31 +4280,31 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>0.0174874532936775</v>
+        <v>-0.1005057949140373</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>4438</v>
+        <v>5534</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>廣越</t>
+          <t>長虹</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>173.6932421871751</v>
+        <v>178.240771971022</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>56.7</v>
+        <v>73.3</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,13 +4315,13 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>40.50211365332815</v>
+        <v>38.58221477615712</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>22.30657845167308</v>
+        <v>16.17922227485474</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>0.1837140938530875</v>
+        <v>0.8600740304657295</v>
       </c>
       <c r="K73" s="2" t="n">
         <v>0</v>
@@ -4333,31 +4333,31 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>0.0482296690875354</v>
+        <v>0.0174874532936775</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>6143</v>
+        <v>4438</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>振曜</t>
+          <t>廣越</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>172.159364220643</v>
+        <v>173.6932421871751</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>81</v>
+        <v>56.7</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,13 +4368,13 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>33.46899048147242</v>
+        <v>40.50211365332815</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>26.29766510420255</v>
+        <v>22.30657845167308</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.5880518134925828</v>
+        <v>0.1837140938530875</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>0</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.0587464727802786</v>
+        <v>0.0482296690875354</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4396,21 +4396,21 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>4414</v>
+        <v>6143</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>如興</t>
+          <t>振曜</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>171.1621627002142</v>
+        <v>172.159364220643</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>8.109999999999999</v>
+        <v>81</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,13 +4421,13 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>40.59865883578896</v>
+        <v>33.46899048147242</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>11.04671932218731</v>
+        <v>26.29766510420255</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>1.064669194445304</v>
+        <v>0.5880518134925828</v>
       </c>
       <c r="K75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>0.0075245557747006</v>
+        <v>0.0587464727802786</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>4572</v>
+        <v>4414</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>駐龍</t>
+          <t>如興</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>163.8285034396278</v>
+        <v>171.1621627002142</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>139</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,13 +4474,13 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>42.0244357305301</v>
+        <v>40.59865883578896</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>11.48872920487935</v>
+        <v>11.04671932218731</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.8278308037344182</v>
+        <v>1.064669194445304</v>
       </c>
       <c r="K76" s="2" t="n">
         <v>0</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.2430393404526393</v>
+        <v>0.0075245557747006</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4502,21 +4502,21 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>5521</v>
+        <v>4572</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>工信</t>
+          <t>駐龍</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>163.7630950926623</v>
+        <v>163.8285034396278</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>10.5</v>
+        <v>139</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,13 +4527,13 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>47.48833843155835</v>
+        <v>42.0244357305301</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>12.56784223695794</v>
+        <v>11.48872920487935</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.462642649631253</v>
+        <v>0.8278308037344182</v>
       </c>
       <c r="K77" s="2" t="n">
         <v>0</v>
@@ -4545,31 +4545,31 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.0110586029491484</v>
+        <v>-0.2430393404526393</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>4737</v>
+        <v>5521</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>華廣</t>
+          <t>工信</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>154.1999338386829</v>
+        <v>163.7630950926623</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>55.6</v>
+        <v>10.5</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,13 +4580,13 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>41.08134351571621</v>
+        <v>47.48833843155835</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>16.96690823552631</v>
+        <v>12.56784223695794</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0.2122420951339727</v>
+        <v>0.462642649631253</v>
       </c>
       <c r="K78" s="2" t="n">
         <v>0</v>
@@ -4598,31 +4598,31 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.2974741847387187</v>
+        <v>-0.0110586029491484</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>4169</v>
+        <v>4737</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>泰宗</t>
+          <t>華廣</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>147.4208261498497</v>
+        <v>154.1999338386829</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>148.5</v>
+        <v>55.6</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,13 +4633,13 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>45.69388008423397</v>
+        <v>41.08134351571621</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>7.53384560424247</v>
+        <v>16.96690823552631</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0.6036704462798932</v>
+        <v>0.2122420951339727</v>
       </c>
       <c r="K79" s="2" t="n">
         <v>0</v>
@@ -4651,31 +4651,31 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>1.21862174081859</v>
+        <v>-0.2974741847387187</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>5283</v>
+        <v>4169</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>禾聯碩</t>
+          <t>泰宗</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>133.3692147582647</v>
+        <v>147.4208261498497</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>52.6</v>
+        <v>148.5</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,13 +4686,13 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>42.98861608699043</v>
+        <v>45.69388008423397</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>15.19705758167092</v>
+        <v>7.53384560424247</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>0.5879074476551605</v>
+        <v>0.6036704462798932</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>0</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-0.0899739854599676</v>
+        <v>1.21862174081859</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4714,21 +4714,21 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>5706</v>
+        <v>5283</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>鳳凰</t>
+          <t>禾聯碩</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>129.1475331497715</v>
+        <v>133.3692147582647</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>43.9</v>
+        <v>52.6</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,13 +4739,13 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>38.17546853089751</v>
+        <v>42.98861608699043</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>18.55368382584277</v>
+        <v>15.19705758167092</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0.8068734014008849</v>
+        <v>0.5879074476551605</v>
       </c>
       <c r="K81" s="2" t="n">
         <v>0</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.0231194652980663</v>
+        <v>-0.0899739854599676</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4767,21 +4767,21 @@
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>4569</v>
+        <v>5706</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>六方科-KY</t>
+          <t>鳳凰</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>112.1871624025854</v>
+        <v>129.1475331497715</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>154</v>
+        <v>43.9</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,13 +4792,13 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>42.20015695642446</v>
+        <v>38.17546853089751</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>16.95597906746356</v>
+        <v>18.55368382584277</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>0.2933248241429343</v>
+        <v>0.8068734014008849</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>0</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.7197012971087138</v>
+        <v>0.0231194652980663</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4820,21 +4820,21 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>5907</v>
+        <v>4569</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>大洋-KY</t>
+          <t>六方科-KY</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>110.5897147625944</v>
+        <v>112.1871624025854</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>4.79</v>
+        <v>154</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,13 +4845,13 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>42.72304175357536</v>
+        <v>42.20015695642446</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>11.57353998141928</v>
+        <v>16.95597906746356</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.258971476259444</v>
+        <v>0.2933248241429343</v>
       </c>
       <c r="K83" s="2" t="n">
         <v>0</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-0.0050558609557016</v>
+        <v>-0.7197012971087138</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>6160</v>
+        <v>5907</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>欣技</t>
+          <t>大洋-KY</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>105.2080274940898</v>
+        <v>110.5897147625944</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>13.9</v>
+        <v>4.79</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,13 +4898,13 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>35.16156081180957</v>
+        <v>42.72304175357536</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>17.53701621150096</v>
+        <v>11.57353998141928</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>0.8097878925657751</v>
+        <v>0.258971476259444</v>
       </c>
       <c r="K84" s="2" t="n">
         <v>0</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.0591248548420993</v>
+        <v>-0.0050558609557016</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4926,21 +4926,21 @@
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>5531</v>
+        <v>6160</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>鄉林</t>
+          <t>欣技</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>92.58928498422046</v>
+        <v>105.2080274940898</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>6.85</v>
+        <v>13.9</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,13 +4951,13 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>34.96509073386741</v>
+        <v>35.16156081180957</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>17.88446806925703</v>
+        <v>17.53701621150096</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.6115448326642708</v>
+        <v>0.8097878925657751</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>0</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-0.0099926029978381</v>
+        <v>-0.0591248548420993</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -4979,21 +4979,21 @@
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>4571</v>
+        <v>5531</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>鈞興-KY</t>
+          <t>鄉林</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>84.91046956713575</v>
+        <v>92.58928498422046</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>152.5</v>
+        <v>6.85</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,13 +5004,13 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>46.27645048438456</v>
+        <v>34.96509073386741</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>14.33741913339222</v>
+        <v>17.88446806925703</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.4160812473714544</v>
+        <v>0.6115448326642708</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>0</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>0.4522751835706655</v>
+        <v>-0.0099926029978381</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5032,52 +5032,105 @@
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
+        <v>4571</v>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>鈞興-KY</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D87" s="2" t="n">
+        <v>84.91046956713575</v>
+      </c>
+      <c r="E87" s="2" t="n">
+        <v>152.5</v>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H87" s="2" t="n">
+        <v>46.27645048438456</v>
+      </c>
+      <c r="I87" s="2" t="n">
+        <v>14.33741913339222</v>
+      </c>
+      <c r="J87" s="2" t="n">
+        <v>0.4160812473714544</v>
+      </c>
+      <c r="K87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M87" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N87" s="2" t="n">
+        <v>0.4522751835706655</v>
+      </c>
+      <c r="O87" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
         <v>5522</v>
       </c>
-      <c r="B87" s="2" t="inlineStr">
+      <c r="B88" s="2" t="inlineStr">
         <is>
           <t>遠雄</t>
         </is>
       </c>
-      <c r="C87" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D87" s="2" t="n">
+      <c r="C88" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D88" s="2" t="n">
         <v>84.1310251618213</v>
       </c>
-      <c r="E87" s="2" t="n">
+      <c r="E88" s="2" t="n">
         <v>60.7</v>
       </c>
-      <c r="F87" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="G87" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H87" s="2" t="n">
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H88" s="2" t="n">
         <v>39.82664315884454</v>
       </c>
-      <c r="I87" s="2" t="n">
+      <c r="I88" s="2" t="n">
         <v>12.92785773895347</v>
       </c>
-      <c r="J87" s="2" t="n">
+      <c r="J88" s="2" t="n">
         <v>0.6332774391347085</v>
       </c>
-      <c r="K87" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L87" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M87" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N87" s="2" t="n">
+      <c r="K88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M88" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N88" s="2" t="n">
         <v>-0.0377134180262009</v>
       </c>
-      <c r="O87" s="2" t="inlineStr">
+      <c r="O88" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, avoid_chase</t>
         </is>

</xml_diff>